<commit_message>
improvements questions and metrics
</commit_message>
<xml_diff>
--- a/public/questions.xlsx
+++ b/public/questions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="170">
   <si>
     <t>category</t>
   </si>
@@ -105,7 +105,7 @@
     <t>¿Cuántas horas tuvo el siglo XX?</t>
   </si>
   <si>
-    <t>¿Cuántos minutos funciona un coche medio en España antes de acabar en el desguace?</t>
+    <t>¿Cuántos minutos se pasa encendido de media un coche en España antes de acabar en el desguace?</t>
   </si>
   <si>
     <t>¿Cuántas horas de Netflix han visto entre todos los españoles entre 2020 y 2025?</t>
@@ -138,7 +138,7 @@
     <t>¿Cuántos kilos pesan entre todos los españoles?</t>
   </si>
   <si>
-    <t>¿Cuántos kilos pesan entre todos los teléfonos móviles de España?</t>
+    <t>¿Cuántos kilos pesan entre todos los teléfonos móviles de España que están encendidos ahora mismo?</t>
   </si>
   <si>
     <t>¿Cuántos kilos pesa la Puerta de Alcalá?</t>
@@ -445,9 +445,6 @@
   </si>
   <si>
     <t>¿Cuántas piezas de LEGO existen actualmente en el mundo (fabricadas desde su inicio)?</t>
-  </si>
-  <si>
-    <t>¿Cuántas veces late el corazón de un ratón de campo en un solo minuto?</t>
   </si>
   <si>
     <t>¿Cuántos litros de agua se evaporan de una piscina olímpica en un día caluroso de agosto?</t>
@@ -8223,195 +8220,193 @@
     </row>
     <row r="3">
       <c r="A3" s="11"/>
-      <c r="B3" s="14" t="s">
-        <v>143</v>
-      </c>
+      <c r="B3" s="14"/>
     </row>
     <row r="4">
       <c r="A4" s="11"/>
       <c r="B4" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11"/>
       <c r="B5" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11"/>
       <c r="B6" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11"/>
       <c r="B7" s="14" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11"/>
       <c r="B8" s="14" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11"/>
       <c r="B9" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11"/>
       <c r="B10" s="14" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11"/>
       <c r="B11" s="14" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11"/>
       <c r="B12" s="14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11"/>
       <c r="B13" s="14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11"/>
       <c r="B14" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11"/>
       <c r="B15" s="14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11"/>
       <c r="B16" s="14" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11"/>
       <c r="B17" s="14" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11"/>
       <c r="B18" s="14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11"/>
       <c r="B19" s="14" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11"/>
       <c r="B20" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="11"/>
       <c r="B21" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11"/>
       <c r="B22" s="14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="11"/>
       <c r="B23" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11"/>
       <c r="B24" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11"/>
       <c r="B25" s="14" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="11"/>
       <c r="B26" s="14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11"/>
       <c r="B27" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11"/>
       <c r="B28" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11"/>
       <c r="B29" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11"/>
       <c r="B30" s="14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>

</xml_diff>